<commit_message>
Updated more names for consistency
</commit_message>
<xml_diff>
--- a/Copy of Lake Trends Revised Updated POR and Percent Change_June25_Revised 04072026.xlsx
+++ b/Copy of Lake Trends Revised Updated POR and Percent Change_June25_Revised 04072026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\WaterQuality\Monitoring\Trends Work 2023\Final Trend Outputs for USE_All Waterbody Types\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://officemgmtentserv-my.sharepoint.com/personal/jordon_henderson_owrb_ok_gov/Documents/Documents/Factsheets_HTML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB8F8A81-B659-460C-97B1-4A36028393DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{AB8F8A81-B659-460C-97B1-4A36028393DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9D38C95-E353-43A7-9918-9A7C988DF3EC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45EE3177-148E-4463-BCC1-B47E3C070BBF}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12897" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12897" uniqueCount="297">
   <si>
     <t>Lake</t>
   </si>
@@ -925,6 +925,15 @@
   <si>
     <t>Jean Neustadt</t>
   </si>
+  <si>
+    <t>Great Salt Plains</t>
+  </si>
+  <si>
+    <t>Lake Hudson (Delaware County)</t>
+  </si>
+  <si>
+    <t>Robert S. Kerr</t>
+  </si>
 </sst>
 </file>
 
@@ -13619,7 +13628,7 @@
     </row>
     <row r="212" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>67</v>
+        <v>294</v>
       </c>
       <c r="B212" t="s">
         <v>11</v>
@@ -13676,7 +13685,7 @@
     </row>
     <row r="213" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>67</v>
+        <v>294</v>
       </c>
       <c r="B213" t="s">
         <v>11</v>
@@ -13736,7 +13745,7 @@
     </row>
     <row r="214" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>67</v>
+        <v>294</v>
       </c>
       <c r="B214" t="s">
         <v>11</v>
@@ -13793,7 +13802,7 @@
     </row>
     <row r="215" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>67</v>
+        <v>294</v>
       </c>
       <c r="B215" t="s">
         <v>11</v>
@@ -13853,7 +13862,7 @@
     </row>
     <row r="216" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>67</v>
+        <v>294</v>
       </c>
       <c r="B216" t="s">
         <v>11</v>
@@ -13910,7 +13919,7 @@
     </row>
     <row r="217" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>67</v>
+        <v>294</v>
       </c>
       <c r="B217" t="s">
         <v>11</v>
@@ -19501,7 +19510,7 @@
     </row>
     <row r="313" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A313" s="5" t="s">
-        <v>208</v>
+        <v>295</v>
       </c>
       <c r="B313" t="s">
         <v>11</v>
@@ -19558,7 +19567,7 @@
     </row>
     <row r="314" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A314" s="5" t="s">
-        <v>208</v>
+        <v>295</v>
       </c>
       <c r="B314" t="s">
         <v>11</v>
@@ -19615,7 +19624,7 @@
     </row>
     <row r="315" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A315" s="5" t="s">
-        <v>208</v>
+        <v>295</v>
       </c>
       <c r="B315" t="s">
         <v>11</v>
@@ -19672,7 +19681,7 @@
     </row>
     <row r="316" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A316" s="5" t="s">
-        <v>208</v>
+        <v>295</v>
       </c>
       <c r="B316" t="s">
         <v>11</v>
@@ -19723,7 +19732,7 @@
     </row>
     <row r="317" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A317" s="5" t="s">
-        <v>208</v>
+        <v>295</v>
       </c>
       <c r="B317" t="s">
         <v>11</v>
@@ -19780,7 +19789,7 @@
     </row>
     <row r="318" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A318" s="5" t="s">
-        <v>208</v>
+        <v>295</v>
       </c>
       <c r="B318" t="s">
         <v>11</v>
@@ -26834,7 +26843,7 @@
     </row>
     <row r="439" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>101</v>
+        <v>296</v>
       </c>
       <c r="B439" t="s">
         <v>11</v>
@@ -26891,7 +26900,7 @@
     </row>
     <row r="440" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>101</v>
+        <v>296</v>
       </c>
       <c r="B440" t="s">
         <v>11</v>
@@ -26951,7 +26960,7 @@
     </row>
     <row r="441" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>101</v>
+        <v>296</v>
       </c>
       <c r="B441" t="s">
         <v>11</v>
@@ -27008,7 +27017,7 @@
     </row>
     <row r="442" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>101</v>
+        <v>296</v>
       </c>
       <c r="B442" t="s">
         <v>11</v>
@@ -27065,7 +27074,7 @@
     </row>
     <row r="443" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>101</v>
+        <v>296</v>
       </c>
       <c r="B443" t="s">
         <v>11</v>
@@ -27122,7 +27131,7 @@
     </row>
     <row r="444" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>101</v>
+        <v>296</v>
       </c>
       <c r="B444" t="s">
         <v>11</v>

</xml_diff>